<commit_message>
Initial PostForge deployment - no secrets
</commit_message>
<xml_diff>
--- a/data/Valencia-Lead-Tracker.xlsx
+++ b/data/Valencia-Lead-Tracker.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P87"/>
+  <dimension ref="A1:P90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4104,7 +4104,7 @@
     </row>
     <row r="81">
       <c r="B81" s="2" t="n">
-        <v>46086.51563790512</v>
+        <v>46086.51563790509</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -4116,9 +4116,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
           <t>Chicago</t>
@@ -4132,7 +4129,6 @@
 Xiomara Solis … See more</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr">
         <is>
           <t>❄️ Cold</t>
@@ -4156,7 +4152,7 @@
     </row>
     <row r="82">
       <c r="B82" s="2" t="n">
-        <v>46086.51563791663</v>
+        <v>46086.51563791667</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -4168,9 +4164,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
           <t>Chicago</t>
@@ -4181,7 +4174,6 @@
           <t>Where was the bitch ?</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr"/>
       <c r="K82" t="inlineStr">
         <is>
           <t>❄️ Cold</t>
@@ -4205,7 +4197,7 @@
     </row>
     <row r="83">
       <c r="B83" s="2" t="n">
-        <v>46086.5156379282</v>
+        <v>46086.51563792824</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -4217,9 +4209,6 @@
           <t>Flooring</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
           <t>Chicago</t>
@@ -4230,7 +4219,6 @@
           <t>You might try one of the vinyl repair kits available at a hardware store. Save you a bundle.</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr">
         <is>
           <t>❄️ Cold</t>
@@ -4254,7 +4242,7 @@
     </row>
     <row r="84">
       <c r="B84" s="2" t="n">
-        <v>46086.51563793988</v>
+        <v>46086.51563793982</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -4266,9 +4254,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
           <t>Chicago</t>
@@ -4279,7 +4264,6 @@
           <t>Hi! I’m a current elementary teacher in the area and tutor grades 1-5 as well. Please let me know ho — Hi! I’m a current elementary teacher in the area and tutor grades 1-5 as well. Please let me know how I can help!</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr">
         <is>
           <t>❄️ Cold</t>
@@ -4303,7 +4287,7 @@
     </row>
     <row r="85">
       <c r="B85" s="2" t="n">
-        <v>46086.5156379515</v>
+        <v>46086.51563795139</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -4315,9 +4299,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
-      <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>Chicago</t>
@@ -4328,7 +4309,6 @@
           <t>I would look into Tree Town Preschool. It’s not a forest school, but it is play based and the kids w — I would look into Tree Town Preschool. It’s not a forest school, but it is play based and the kids will spend time outside exp… See more</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr">
         <is>
           <t>❄️ Cold</t>
@@ -4352,7 +4332,7 @@
     </row>
     <row r="86">
       <c r="B86" s="2" t="n">
-        <v>46086.51563796298</v>
+        <v>46086.51563796296</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -4364,9 +4344,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>Chicago</t>
@@ -4377,7 +4354,6 @@
           <t>What's the web site to apply at?.</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr">
         <is>
           <t>❄️ Cold</t>
@@ -4401,7 +4377,7 @@
     </row>
     <row r="87">
       <c r="B87" s="2" t="n">
-        <v>46086.51563796298</v>
+        <v>46086.51563796296</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -4413,9 +4389,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
           <t>Chicago</t>
@@ -4426,7 +4399,6 @@
           <t>Can you do an estimate to replace the glass on a 5'×4' picture window at a house in Wood Dale?</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr">
         <is>
           <t>❄️ Cold</t>
@@ -4445,6 +4417,154 @@
       <c r="P87" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/ElmwoodParkIL60707/posts/26211425471844604/</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="2" t="n">
+        <v>46086.62815994504</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Make sure the oil doesn’t look brown like it’s mixed with antifreeze type of thing</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/464809784881517/posts/1682843846411432/</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="2" t="n">
+        <v>46086.62815995661</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>If youre looking for the big ones 
+Stock 'n Save carries them</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>⚡ Warm</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/belmontcragincommunity/posts/2147957429295699/</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="2" t="n">
+        <v>46086.6281601478</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>What kind of phone do you have? You can transfer photos from phone to Google photos ( Cloud)..</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>⚡ Warm</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/148056482809454/posts/1622155568732864/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 2: Auto-Pilot Scheduler - recurring schedules + auto-generation + approval workflow
</commit_message>
<xml_diff>
--- a/data/Valencia-Lead-Tracker.xlsx
+++ b/data/Valencia-Lead-Tracker.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P90"/>
+  <dimension ref="A1:P103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4422,7 +4422,7 @@
     </row>
     <row r="88">
       <c r="B88" s="2" t="n">
-        <v>46086.62815994504</v>
+        <v>46086.62815994213</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -4434,9 +4434,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>Chicago</t>
@@ -4447,7 +4444,6 @@
           <t>Make sure the oil doesn’t look brown like it’s mixed with antifreeze type of thing</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr">
         <is>
           <t>❄️ Cold</t>
@@ -4471,7 +4467,7 @@
     </row>
     <row r="89">
       <c r="B89" s="2" t="n">
-        <v>46086.62815995661</v>
+        <v>46086.6281599537</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -4483,9 +4479,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
           <t>Chicago</t>
@@ -4497,7 +4490,6 @@
 Stock 'n Save carries them</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
           <t>⚡ Warm</t>
@@ -4521,7 +4513,7 @@
     </row>
     <row r="90">
       <c r="B90" s="2" t="n">
-        <v>46086.6281601478</v>
+        <v>46086.62816015046</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -4533,9 +4525,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>Chicago</t>
@@ -4546,7 +4535,6 @@
           <t>What kind of phone do you have? You can transfer photos from phone to Google photos ( Cloud)..</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr">
         <is>
           <t>⚡ Warm</t>
@@ -4565,6 +4553,619 @@
       <c r="P90" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/148056482809454/posts/1622155568732864/</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="2" t="n">
+        <v>46087.54509413194</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Would you be interested in a live in Nanny?</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/148056482809454/posts/1623389035276184/</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="2" t="n">
+        <v>46087.54509414352</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Versailles on the Lakes Oakbrook will do short term.</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/elmhurstnews/posts/26212376125040725/</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="2" t="n">
+        <v>46087.54509414352</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Mariela Pineda disculpe si tiene huanzontles ? Estoy saliendo del trabajo y quiero ir por unos porfa — Mariela Pineda disculpe si tiene huanzontles ? Estoy saliendo del trabajo y quiero ir por unos porfavor gracias</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1463608113861939/posts/4424940874395300/</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" s="2" t="n">
+        <v>46087.6280478125</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Just up the road in Lincolnshire is Kossof Salon Spa. Did mani/pedi myself twice in the last month.  — Just up the road in Lincolnshire is Kossof Salon Spa. Did mani/pedi myself twice in the last month. They are fantastic.</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/thenorthbrookneighbors/posts/1861335977855352/</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" s="2" t="n">
+        <v>46087.62804784723</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Jewel’s is really good.</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/elmhurstnews/posts/26218789141066090/</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" s="2" t="n">
+        <v>46087.62804787037</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Meet your admin team: Alex Hodorovych</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1463608113861939/posts/4425072367715484/</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="2" t="n">
+        <v>46088.72848677141</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>You need a wax ring. I’d bet cost to change it that solves your issue</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>⚡ Warm</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/470730068060176/posts/1434561341677039/</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" s="2" t="n">
+        <v>46088.72848691633</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>I definitely wanna see a follow up on this. They’re not gonna be happy about the visits that they’re — I definitely wanna see a follow up on this. They’re not gonna be happy about the visits that they’re gonna get lol if they tho… See more</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/belmontcragincommunity/posts/2150142429077199/</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="2" t="n">
+        <v>46088.72848693372</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Where can we sign up!! Also is there a cap in your class?</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/belmontcragincommunity/posts/2149752005782908/</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" s="2" t="n">
+        <v>46088.72848693372</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>GarageExperts of Chicagoland best around … See more</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/elmhurstnews/posts/26228241286787542/</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="2" t="n">
+        <v>46088.72848695135</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>salvation army trailer on Summit east side a few blocks south of roosevelt. at the church too just s — salvation army trailer on Summit east side a few blocks south of roosevelt. at the church too just south of trailer</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/elmhurstnews/posts/26223084470636557/</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" s="2" t="n">
+        <v>46088.72848695135</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>All postal service everywhere</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/elmhurstnews/posts/26221519330793071/</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" s="2" t="n">
+        <v>46088.72848696297</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>I used Apex and very happy with there work.</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>❄️ Cold</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/878691372244191/posts/26195442290142417/</t>
         </is>
       </c>
     </row>

</xml_diff>